<commit_message>
upd: rewrite the target to target distances with itertools library add: issue log add: target to target distances calculations sheet in excel ref: create directory for temp spare modules
</commit_message>
<xml_diff>
--- a/codingame/competitions/02_pacman/pacman.xlsx
+++ b/codingame/competitions/02_pacman/pacman.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\30_git\10_my_code\02_coding-challenges\codingame\competitions\02_pacman\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0675E88-07D3-4A3D-8C33-E4041CB13C81}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82AF7A34-8FBA-4051-A4E8-09BDC9C7EBB0}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="16530" yWindow="4020" windowWidth="20310" windowHeight="14040" xr2:uid="{806FAAE1-1476-49A1-B2F5-955C11E74D2D}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="s2s distances" sheetId="2" r:id="rId1"/>
+    <sheet name="p2s distances" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="12">
   <si>
     <t>x</t>
   </si>
@@ -96,7 +97,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -119,11 +120,40 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -135,6 +165,21 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -450,6 +495,273 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99B8CE4E-51F9-4FD8-96EF-9C14C9AE9367}">
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="3" width="7.140625" customWidth="1"/>
+    <col min="4" max="4" width="4.140625" customWidth="1"/>
+    <col min="5" max="9" width="7.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="1"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" s="1"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="3">
+        <v>8</v>
+      </c>
+      <c r="F3" s="3">
+        <v>11</v>
+      </c>
+      <c r="G3" s="3">
+        <v>19</v>
+      </c>
+      <c r="H3" s="3">
+        <v>22</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="3">
+        <v>9</v>
+      </c>
+      <c r="F4" s="3">
+        <v>10</v>
+      </c>
+      <c r="G4" s="3">
+        <v>10</v>
+      </c>
+      <c r="H4" s="3">
+        <v>9</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="3">
+        <v>8</v>
+      </c>
+      <c r="C6" s="3">
+        <v>9</v>
+      </c>
+      <c r="D6" s="1"/>
+      <c r="E6" s="3">
+        <f t="shared" ref="E6:G9" si="0">ABS($B6-E$3) + ABS($C6-E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="3">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="G6" s="3">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="H6" s="3"/>
+      <c r="I6" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="3">
+        <v>11</v>
+      </c>
+      <c r="C7" s="3">
+        <v>10</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="E7" s="3">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="F7" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G7" s="3">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="H7" s="3"/>
+      <c r="I7" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="3">
+        <v>19</v>
+      </c>
+      <c r="C8" s="3">
+        <v>10</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="3">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="F8" s="3">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="G8" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H8" s="3"/>
+      <c r="I8" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="3">
+        <v>22</v>
+      </c>
+      <c r="C9" s="3">
+        <v>9</v>
+      </c>
+      <c r="D9" s="1"/>
+      <c r="E9" s="3">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="F9" s="3">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="G9" s="3">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="H9" s="3"/>
+      <c r="I9" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="1"/>
+      <c r="B10" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="E10" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I10" s="1"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="1"/>
+      <c r="B11" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C11" s="5"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="E1:H1"/>
+    <mergeCell ref="E11:H11"/>
+  </mergeCells>
+  <conditionalFormatting sqref="E6:H9">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7B64D38-74B5-462B-A6AE-04115298AA8B}">
   <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -464,11 +776,11 @@
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
       <c r="H1" s="1"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -663,16 +975,16 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="4"/>
+      <c r="C11" s="5"/>
       <c r="D11" s="1"/>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
       <c r="H11" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
first draft of cluster
</commit_message>
<xml_diff>
--- a/codingame/competitions/02_pacman/pacman.xlsx
+++ b/codingame/competitions/02_pacman/pacman.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\30_git\10_my_code\02_coding-challenges\codingame\competitions\02_pacman\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82AF7A34-8FBA-4051-A4E8-09BDC9C7EBB0}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{759811A4-15BE-4CF7-8985-9802597751B9}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16530" yWindow="4020" windowWidth="20310" windowHeight="14040" xr2:uid="{806FAAE1-1476-49A1-B2F5-955C11E74D2D}"/>
+    <workbookView xWindow="1680" yWindow="4110" windowWidth="10770" windowHeight="10095" xr2:uid="{806FAAE1-1476-49A1-B2F5-955C11E74D2D}"/>
   </bookViews>
   <sheets>
     <sheet name="s2s distances" sheetId="2" r:id="rId1"/>
@@ -97,7 +97,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -120,40 +120,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -168,18 +139,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -509,12 +468,12 @@
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
       <c r="I1" s="1"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -601,7 +560,7 @@
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="3">
-        <f t="shared" ref="E6:G9" si="0">ABS($B6-E$3) + ABS($C6-E$4)</f>
+        <f t="shared" ref="E6:H9" si="0">ABS($B6-E$3) + ABS($C6-E$4)</f>
         <v>0</v>
       </c>
       <c r="F6" s="3">
@@ -612,7 +571,10 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="H6" s="3"/>
+      <c r="H6" s="3">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
       <c r="I6" s="4" t="s">
         <v>8</v>
       </c>
@@ -640,7 +602,10 @@
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="H7" s="3"/>
+      <c r="H7" s="3">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
       <c r="I7" s="4" t="s">
         <v>7</v>
       </c>
@@ -668,7 +633,10 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="3"/>
+      <c r="H8" s="3">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
       <c r="I8" s="4" t="s">
         <v>9</v>
       </c>
@@ -696,7 +664,10 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="H9" s="3"/>
+      <c r="H9" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="I9" s="4" t="s">
         <v>10</v>
       </c>
@@ -731,12 +702,12 @@
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="1"/>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
       <c r="I11" s="1"/>
     </row>
   </sheetData>
@@ -758,6 +729,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
add: max peace turns
</commit_message>
<xml_diff>
--- a/codingame/competitions/02_pacman/pacman.xlsx
+++ b/codingame/competitions/02_pacman/pacman.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\30_git\10_my_code\02_coding-challenges\codingame\competitions\02_pacman\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{759811A4-15BE-4CF7-8985-9802597751B9}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30A647BD-5FDC-4152-BCDD-CD6DD710B617}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1680" yWindow="4110" windowWidth="10770" windowHeight="10095" xr2:uid="{806FAAE1-1476-49A1-B2F5-955C11E74D2D}"/>
+    <workbookView xWindow="12795" yWindow="4035" windowWidth="15060" windowHeight="14895" activeTab="2" xr2:uid="{806FAAE1-1476-49A1-B2F5-955C11E74D2D}"/>
   </bookViews>
   <sheets>
     <sheet name="s2s distances" sheetId="2" r:id="rId1"/>
     <sheet name="p2s distances" sheetId="1" r:id="rId2"/>
+    <sheet name="heuristic function" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="16">
   <si>
     <t>x</t>
   </si>
@@ -69,6 +70,18 @@
   <si>
     <t>Manh. distances</t>
   </si>
+  <si>
+    <t>count</t>
+  </si>
+  <si>
+    <t>empty</t>
+  </si>
+  <si>
+    <t>total</t>
+  </si>
+  <si>
+    <t>density</t>
+  </si>
 </sst>
 </file>
 
@@ -83,7 +96,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -93,6 +106,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -124,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -141,6 +166,14 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -979,4 +1012,519 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4C6B770-3647-439D-A74C-C787D5A82A3B}">
+  <dimension ref="A1:E25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="6">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6">
+        <v>0</v>
+      </c>
+      <c r="C2" s="7">
+        <f t="shared" ref="C2:C8" si="0">A2+B2</f>
+        <v>1</v>
+      </c>
+      <c r="D2" s="8">
+        <f t="shared" ref="D2:D8" si="1">A2/C2</f>
+        <v>1</v>
+      </c>
+      <c r="E2" s="8">
+        <f>A2*D2^2</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" s="9">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="D3" s="10">
+        <f t="shared" si="1"/>
+        <v>0.5</v>
+      </c>
+      <c r="E3" s="10">
+        <f t="shared" ref="E3:E25" si="2">A3*D3^2</f>
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" s="9">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="D4" s="10">
+        <f t="shared" si="1"/>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="E4" s="10">
+        <f t="shared" si="2"/>
+        <v>0.1111111111111111</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5" s="9">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="D5" s="10">
+        <f t="shared" si="1"/>
+        <v>0.25</v>
+      </c>
+      <c r="E5" s="10">
+        <f t="shared" si="2"/>
+        <v>6.25E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>1</v>
+      </c>
+      <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="C6" s="9">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="D6" s="10">
+        <f t="shared" si="1"/>
+        <v>0.2</v>
+      </c>
+      <c r="E6" s="10">
+        <f t="shared" si="2"/>
+        <v>4.0000000000000008E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>1</v>
+      </c>
+      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7" s="9">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="D7" s="10">
+        <f t="shared" si="1"/>
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="E7" s="10">
+        <f t="shared" si="2"/>
+        <v>2.7777777777777776E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>1</v>
+      </c>
+      <c r="B8">
+        <v>6</v>
+      </c>
+      <c r="C8" s="9">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="D8" s="10">
+        <f t="shared" si="1"/>
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="E8" s="10">
+        <f t="shared" si="2"/>
+        <v>2.0408163265306121E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="11">
+        <v>2</v>
+      </c>
+      <c r="B9" s="12">
+        <v>0</v>
+      </c>
+      <c r="C9" s="12">
+        <f>A9+B9</f>
+        <v>2</v>
+      </c>
+      <c r="D9" s="13">
+        <f>A9/C9</f>
+        <v>1</v>
+      </c>
+      <c r="E9" s="13">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>2</v>
+      </c>
+      <c r="B10" s="9">
+        <v>1</v>
+      </c>
+      <c r="C10" s="9">
+        <f t="shared" ref="C10:C25" si="3">A10+B10</f>
+        <v>3</v>
+      </c>
+      <c r="D10" s="10">
+        <f t="shared" ref="D10:D25" si="4">A10/C10</f>
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="E10" s="10">
+        <f t="shared" si="2"/>
+        <v>0.88888888888888884</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>2</v>
+      </c>
+      <c r="B11" s="9">
+        <v>2</v>
+      </c>
+      <c r="C11" s="9">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="D11" s="10">
+        <f t="shared" si="4"/>
+        <v>0.5</v>
+      </c>
+      <c r="E11" s="10">
+        <f t="shared" si="2"/>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>2</v>
+      </c>
+      <c r="B12" s="9">
+        <v>3</v>
+      </c>
+      <c r="C12" s="9">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="D12" s="10">
+        <f t="shared" si="4"/>
+        <v>0.4</v>
+      </c>
+      <c r="E12" s="10">
+        <f t="shared" si="2"/>
+        <v>0.32000000000000006</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>2</v>
+      </c>
+      <c r="B13" s="9">
+        <v>4</v>
+      </c>
+      <c r="C13" s="9">
+        <f t="shared" si="3"/>
+        <v>6</v>
+      </c>
+      <c r="D13" s="10">
+        <f t="shared" si="4"/>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="E13" s="10">
+        <f t="shared" si="2"/>
+        <v>0.22222222222222221</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>3</v>
+      </c>
+      <c r="B14" s="9">
+        <v>0</v>
+      </c>
+      <c r="C14" s="9">
+        <f t="shared" si="3"/>
+        <v>3</v>
+      </c>
+      <c r="D14" s="10">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="E14" s="10">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>3</v>
+      </c>
+      <c r="B15" s="9">
+        <f>B14+1</f>
+        <v>1</v>
+      </c>
+      <c r="C15" s="9">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="D15" s="10">
+        <f t="shared" si="4"/>
+        <v>0.75</v>
+      </c>
+      <c r="E15" s="10">
+        <f t="shared" si="2"/>
+        <v>1.6875</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>3</v>
+      </c>
+      <c r="B16" s="9">
+        <f t="shared" ref="B16:B25" si="5">B15+1</f>
+        <v>2</v>
+      </c>
+      <c r="C16" s="9">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="D16" s="10">
+        <f t="shared" si="4"/>
+        <v>0.6</v>
+      </c>
+      <c r="E16" s="10">
+        <f t="shared" si="2"/>
+        <v>1.08</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>3</v>
+      </c>
+      <c r="B17" s="9">
+        <f t="shared" si="5"/>
+        <v>3</v>
+      </c>
+      <c r="C17" s="9">
+        <f t="shared" si="3"/>
+        <v>6</v>
+      </c>
+      <c r="D17" s="10">
+        <f t="shared" si="4"/>
+        <v>0.5</v>
+      </c>
+      <c r="E17" s="10">
+        <f t="shared" si="2"/>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>3</v>
+      </c>
+      <c r="B18" s="9">
+        <f t="shared" si="5"/>
+        <v>4</v>
+      </c>
+      <c r="C18" s="9">
+        <f t="shared" si="3"/>
+        <v>7</v>
+      </c>
+      <c r="D18" s="10">
+        <f t="shared" si="4"/>
+        <v>0.42857142857142855</v>
+      </c>
+      <c r="E18" s="10">
+        <f t="shared" si="2"/>
+        <v>0.55102040816326525</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>3</v>
+      </c>
+      <c r="B19" s="9">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="C19" s="9">
+        <f t="shared" si="3"/>
+        <v>8</v>
+      </c>
+      <c r="D19" s="10">
+        <f t="shared" si="4"/>
+        <v>0.375</v>
+      </c>
+      <c r="E19" s="10">
+        <f t="shared" si="2"/>
+        <v>0.421875</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>3</v>
+      </c>
+      <c r="B20" s="9">
+        <f t="shared" si="5"/>
+        <v>6</v>
+      </c>
+      <c r="C20" s="9">
+        <f t="shared" si="3"/>
+        <v>9</v>
+      </c>
+      <c r="D20" s="10">
+        <f t="shared" si="4"/>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="E20" s="10">
+        <f t="shared" si="2"/>
+        <v>0.33333333333333331</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>3</v>
+      </c>
+      <c r="B21" s="9">
+        <f t="shared" si="5"/>
+        <v>7</v>
+      </c>
+      <c r="C21" s="9">
+        <f t="shared" si="3"/>
+        <v>10</v>
+      </c>
+      <c r="D21" s="10">
+        <f t="shared" si="4"/>
+        <v>0.3</v>
+      </c>
+      <c r="E21" s="10">
+        <f t="shared" si="2"/>
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>3</v>
+      </c>
+      <c r="B22" s="9">
+        <f t="shared" si="5"/>
+        <v>8</v>
+      </c>
+      <c r="C22" s="9">
+        <f t="shared" si="3"/>
+        <v>11</v>
+      </c>
+      <c r="D22" s="10">
+        <f t="shared" si="4"/>
+        <v>0.27272727272727271</v>
+      </c>
+      <c r="E22" s="10">
+        <f t="shared" si="2"/>
+        <v>0.22314049586776857</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>3</v>
+      </c>
+      <c r="B23" s="9">
+        <f t="shared" si="5"/>
+        <v>9</v>
+      </c>
+      <c r="C23" s="9">
+        <f t="shared" si="3"/>
+        <v>12</v>
+      </c>
+      <c r="D23" s="10">
+        <f t="shared" si="4"/>
+        <v>0.25</v>
+      </c>
+      <c r="E23" s="10">
+        <f t="shared" si="2"/>
+        <v>0.1875</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>3</v>
+      </c>
+      <c r="B24" s="9">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="C24" s="9">
+        <f t="shared" si="3"/>
+        <v>13</v>
+      </c>
+      <c r="D24" s="10">
+        <f t="shared" si="4"/>
+        <v>0.23076923076923078</v>
+      </c>
+      <c r="E24" s="10">
+        <f t="shared" si="2"/>
+        <v>0.15976331360946749</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>3</v>
+      </c>
+      <c r="B25" s="9">
+        <f t="shared" si="5"/>
+        <v>11</v>
+      </c>
+      <c r="C25" s="9">
+        <f t="shared" si="3"/>
+        <v>14</v>
+      </c>
+      <c r="D25" s="10">
+        <f t="shared" si="4"/>
+        <v>0.21428571428571427</v>
+      </c>
+      <c r="E25" s="10">
+        <f t="shared" si="2"/>
+        <v>0.13775510204081631</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>